<commit_message>
Add cost-loading columns to self-employed payment reports
Both the flat and the entity-grouped workbooks now carry four derived
columns off the 2026 monthly run-rate: 4dev platform fee (3%), the
Singapore entity gross-up (divide by 0.975), the 6% NPD tax, and a
combined monthly cost. Rates live in editable assumption cells so the
whole sheet and the planning block recalculate when they change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wo4Lmevz8VeqLa4QdqkBF
</commit_message>
<xml_diff>
--- a/СЗ_длительные_выплаты_2022-2026.xlsx
+++ b/СЗ_длительные_выплаты_2022-2026.xlsx
@@ -10,7 +10,7 @@
     <sheet name="СЗ 2022-2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'СЗ 2022-2026'!$A$5:$O$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'СЗ 2022-2026'!$A$10:$S$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;(#,##0);-"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="#,##0;(#,##0);-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,18 +43,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000000FF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,6 +52,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="000000FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -73,8 +69,24 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -101,7 +113,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCE6F1"/>
+        <fgColor rgb="00B4C6E7"/>
       </patternFill>
     </fill>
     <fill>
@@ -136,38 +148,45 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -533,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:S47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -551,6 +570,10 @@
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -577,1465 +600,1880 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Выплат в 2026 (мес.):</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
+          <t>ДОПУЩЕНИЯ (синие ячейки — можно менять, всё пересчитается):</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Выплат в 2026 (мес.)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>← допущение: в 2026 прошло 7 выплат (16.01, 13.02, 13.03, 15.04, 15.05, 15.06, 15.07)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>← 16.01, 13.02, 13.03, 15.04, 15.05, 15.06, 15.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Комиссия платформы 4dev</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>← начисляется сверху на среднемесячную</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Сбор ЮЛ Сингапура</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>← среднемесячная делится на (1 − ставка) = 0,975</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Ставка НПД</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>← начисляется сверху на среднемесячную</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>№</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>ФИО</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Проект</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>ЮЛ</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Ставка НПД</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Период выплат</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Лет</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="M10" s="7" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N10" s="7" t="inlineStr">
         <is>
           <t>Итого 2022–2026</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="O10" s="7" t="inlineStr">
         <is>
           <t>Среднемес. выплата 2026</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="P10" s="7" t="inlineStr">
+        <is>
+          <t>Комиссия 4dev 3%</t>
+        </is>
+      </c>
+      <c r="Q10" s="7" t="inlineStr">
+        <is>
+          <t>Со сбором ЮЛ Сингапур (÷0,975)</t>
+        </is>
+      </c>
+      <c r="R10" s="7" t="inlineStr">
+        <is>
+          <t>С НПД +6%</t>
+        </is>
+      </c>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>ИТОГО к оплате в месяц</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Глубокая Яна Ярославовна</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="H11" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I11" s="10" t="n">
         <v>74734</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J11" s="10" t="n">
         <v>1277373</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="K11" s="10" t="n">
         <v>2001199</v>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="L11" s="10" t="n">
         <v>2541224</v>
       </c>
-      <c r="M6" s="8" t="n">
+      <c r="M11" s="10" t="n">
         <v>1468449.18</v>
       </c>
-      <c r="N6" s="9">
-        <f>SUM(I6:M6)</f>
-        <v/>
-      </c>
-      <c r="O6" s="10">
-        <f>M6/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="n">
+      <c r="N11" s="11">
+        <f>SUM(I11:M11)</f>
+        <v/>
+      </c>
+      <c r="O11" s="11">
+        <f>M11/$C$5</f>
+        <v/>
+      </c>
+      <c r="P11" s="12">
+        <f>O11*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q11" s="12">
+        <f>O11/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R11" s="12">
+        <f>O11*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S11" s="13">
+        <f>O11/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Высочинский Даниил Сергеевич</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ОСП)</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G7" s="11" t="inlineStr">
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H7" s="11" t="n">
+      <c r="H12" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I12" s="16" t="n">
         <v>43489</v>
       </c>
-      <c r="J7" s="13" t="n">
+      <c r="J12" s="16" t="n">
         <v>715306.13</v>
       </c>
-      <c r="K7" s="13" t="n">
+      <c r="K12" s="16" t="n">
         <v>1582317</v>
       </c>
-      <c r="L7" s="13" t="n">
+      <c r="L12" s="16" t="n">
         <v>1778297</v>
       </c>
-      <c r="M7" s="13" t="n">
+      <c r="M12" s="16" t="n">
         <v>1146293</v>
       </c>
-      <c r="N7" s="14">
-        <f>SUM(I7:M7)</f>
-        <v/>
-      </c>
-      <c r="O7" s="15">
-        <f>M7/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="N12" s="17">
+        <f>SUM(I12:M12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="17">
+        <f>M12/$C$5</f>
+        <v/>
+      </c>
+      <c r="P12" s="18">
+        <f>O12*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q12" s="18">
+        <f>O12/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R12" s="18">
+        <f>O12*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S12" s="19">
+        <f>O12/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>Дроздова Мария Глебовна</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>ТФМ (ОСП)</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="H13" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I13" s="10" t="n">
         <v>41064</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J13" s="10" t="n">
         <v>637553</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="K13" s="10" t="n">
         <v>1442457</v>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="L13" s="10" t="n">
         <v>1784722</v>
       </c>
-      <c r="M8" s="8" t="n">
+      <c r="M13" s="10" t="n">
         <v>1222167</v>
       </c>
-      <c r="N8" s="9">
-        <f>SUM(I8:M8)</f>
-        <v/>
-      </c>
-      <c r="O8" s="10">
-        <f>M8/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="n">
+      <c r="N13" s="11">
+        <f>SUM(I13:M13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="11">
+        <f>M13/$C$5</f>
+        <v/>
+      </c>
+      <c r="P13" s="12">
+        <f>O13*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q13" s="12">
+        <f>O13/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R13" s="12">
+        <f>O13*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S13" s="13">
+        <f>O13/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Грудинин Алексей Сергеевич</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
+      <c r="G14" s="14" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="H14" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="I9" s="13" t="n">
+      <c r="I14" s="16" t="n">
         <v>267577.88</v>
       </c>
-      <c r="J9" s="13" t="n">
+      <c r="J14" s="16" t="n">
         <v>960405.97</v>
       </c>
-      <c r="K9" s="13" t="n">
+      <c r="K14" s="16" t="n">
         <v>1372957.36</v>
       </c>
-      <c r="L9" s="13" t="n">
+      <c r="L14" s="16" t="n">
         <v>1558585.08</v>
       </c>
-      <c r="M9" s="13" t="n">
+      <c r="M14" s="16" t="n">
         <v>938053.12</v>
       </c>
-      <c r="N9" s="14">
-        <f>SUM(I9:M9)</f>
-        <v/>
-      </c>
-      <c r="O9" s="15">
-        <f>M9/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="N14" s="17">
+        <f>SUM(I14:M14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="17">
+        <f>M14/$C$5</f>
+        <v/>
+      </c>
+      <c r="P14" s="18">
+        <f>O14*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q14" s="18">
+        <f>O14/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R14" s="18">
+        <f>O14*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S14" s="19">
+        <f>O14/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Кузьмина Елена Игоревна</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>ТФМ (ОСП)</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="H15" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I15" s="10" t="n">
         <v>59574</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J15" s="10" t="n">
         <v>100638</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="K15" s="10" t="n">
         <v>1253297</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="L15" s="10" t="n">
         <v>115745</v>
       </c>
-      <c r="M10" s="8" t="n">
+      <c r="M15" s="10" t="n">
         <v>1062722</v>
       </c>
-      <c r="N10" s="9">
-        <f>SUM(I10:M10)</f>
-        <v/>
-      </c>
-      <c r="O10" s="10">
-        <f>M10/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="N15" s="11">
+        <f>SUM(I15:M15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="11">
+        <f>M15/$C$5</f>
+        <v/>
+      </c>
+      <c r="P15" s="12">
+        <f>O15*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q15" s="12">
+        <f>O15/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R15" s="12">
+        <f>O15*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S15" s="13">
+        <f>O15/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Репетенко Инна Эдуардовна</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ОРБ)</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E16" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G11" s="11" t="inlineStr">
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H16" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="I11" s="13" t="n">
+      <c r="I16" s="16" t="n">
         <v>112190</v>
       </c>
-      <c r="J11" s="13" t="n">
+      <c r="J16" s="16" t="n">
         <v>246600</v>
       </c>
-      <c r="K11" s="13" t="n">
+      <c r="K16" s="16" t="n">
         <v>415655.93</v>
       </c>
-      <c r="L11" s="13" t="n">
+      <c r="L16" s="16" t="n">
         <v>142973.52</v>
       </c>
-      <c r="M11" s="13" t="n">
+      <c r="M16" s="16" t="n">
         <v>905821.35</v>
       </c>
-      <c r="N11" s="14">
-        <f>SUM(I11:M11)</f>
-        <v/>
-      </c>
-      <c r="O11" s="15">
-        <f>M11/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="N16" s="17">
+        <f>SUM(I16:M16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="17">
+        <f>M16/$C$5</f>
+        <v/>
+      </c>
+      <c r="P16" s="18">
+        <f>O16*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q16" s="18">
+        <f>O16/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R16" s="18">
+        <f>O16*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S16" s="19">
+        <f>O16/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Злобин Николай Алексеевич</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D17" s="8" t="inlineStr">
         <is>
           <t>ИП МТ</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F17" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n">
+      <c r="H17" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I17" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="J17" s="10" t="n">
         <v>231383</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="K17" s="10" t="n">
         <v>2343163.34</v>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="L17" s="10" t="n">
         <v>2601170</v>
       </c>
-      <c r="M12" s="8" t="n">
+      <c r="M17" s="10" t="n">
         <v>1832861.81</v>
       </c>
-      <c r="N12" s="9">
-        <f>SUM(I12:M12)</f>
-        <v/>
-      </c>
-      <c r="O12" s="10">
-        <f>M12/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="N17" s="11">
+        <f>SUM(I17:M17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="11">
+        <f>M17/$C$5</f>
+        <v/>
+      </c>
+      <c r="P17" s="12">
+        <f>O17*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q17" s="12">
+        <f>O17/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R17" s="12">
+        <f>O17*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S17" s="13">
+        <f>O17/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Жиркова Валентина Александровна</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G13" s="11" t="inlineStr">
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H13" s="11" t="n">
+      <c r="H18" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I13" s="13" t="n">
+      <c r="I18" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="13" t="n">
+      <c r="J18" s="16" t="n">
         <v>257222.24</v>
       </c>
-      <c r="K13" s="13" t="n">
+      <c r="K18" s="16" t="n">
         <v>1497661</v>
       </c>
-      <c r="L13" s="13" t="n">
+      <c r="L18" s="16" t="n">
         <v>2201639.5</v>
       </c>
-      <c r="M13" s="13" t="n">
+      <c r="M18" s="16" t="n">
         <v>1656517.19</v>
       </c>
-      <c r="N13" s="14">
-        <f>SUM(I13:M13)</f>
-        <v/>
-      </c>
-      <c r="O13" s="15">
-        <f>M13/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="N18" s="17">
+        <f>SUM(I18:M18)</f>
+        <v/>
+      </c>
+      <c r="O18" s="17">
+        <f>M18/$C$5</f>
+        <v/>
+      </c>
+      <c r="P18" s="18">
+        <f>O18*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q18" s="18">
+        <f>O18/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R18" s="18">
+        <f>O18*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S18" s="19">
+        <f>O18/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Гатиатуллина Марина Эдуардовна</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H14" s="6" t="n">
+      <c r="H19" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I19" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J19" s="10" t="n">
         <v>269105.17</v>
       </c>
-      <c r="K14" s="8" t="n">
+      <c r="K19" s="10" t="n">
         <v>1743298</v>
       </c>
-      <c r="L14" s="8" t="n">
+      <c r="L19" s="10" t="n">
         <v>1991245.01</v>
       </c>
-      <c r="M14" s="8" t="n">
+      <c r="M19" s="10" t="n">
         <v>1192011.1</v>
       </c>
-      <c r="N14" s="9">
-        <f>SUM(I14:M14)</f>
-        <v/>
-      </c>
-      <c r="O14" s="10">
-        <f>M14/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="N19" s="11">
+        <f>SUM(I19:M19)</f>
+        <v/>
+      </c>
+      <c r="O19" s="11">
+        <f>M19/$C$5</f>
+        <v/>
+      </c>
+      <c r="P19" s="12">
+        <f>O19*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q19" s="12">
+        <f>O19/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R19" s="12">
+        <f>O19*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S19" s="13">
+        <f>O19/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Оглезнева Полина Сергеевна</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ОСП)</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D20" s="14" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
+      <c r="E20" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G15" s="11" t="inlineStr">
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H20" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I15" s="13" t="n">
+      <c r="I20" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J15" s="13" t="n">
+      <c r="J20" s="16" t="n">
         <v>140852</v>
       </c>
-      <c r="K15" s="13" t="n">
+      <c r="K20" s="16" t="n">
         <v>205851</v>
       </c>
-      <c r="L15" s="13" t="n">
+      <c r="L20" s="16" t="n">
         <v>2326991</v>
       </c>
-      <c r="M15" s="13" t="n">
+      <c r="M20" s="16" t="n">
         <v>1574518</v>
       </c>
-      <c r="N15" s="14">
-        <f>SUM(I15:M15)</f>
-        <v/>
-      </c>
-      <c r="O15" s="15">
-        <f>M15/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n">
+      <c r="N20" s="17">
+        <f>SUM(I20:M20)</f>
+        <v/>
+      </c>
+      <c r="O20" s="17">
+        <f>M20/$C$5</f>
+        <v/>
+      </c>
+      <c r="P20" s="18">
+        <f>O20*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q20" s="18">
+        <f>O20/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R20" s="18">
+        <f>O20*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S20" s="19">
+        <f>O20/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Бобрышева Татьяна Сергеевна</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H16" s="6" t="n">
+      <c r="H21" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I21" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="8" t="n">
+      <c r="J21" s="10" t="n">
         <v>554372.52</v>
       </c>
-      <c r="K16" s="8" t="n">
+      <c r="K21" s="10" t="n">
         <v>1016796.76</v>
       </c>
-      <c r="L16" s="8" t="n">
+      <c r="L21" s="10" t="n">
         <v>1505710.52</v>
       </c>
-      <c r="M16" s="8" t="n">
+      <c r="M21" s="10" t="n">
         <v>1082430.98</v>
       </c>
-      <c r="N16" s="9">
-        <f>SUM(I16:M16)</f>
-        <v/>
-      </c>
-      <c r="O16" s="10">
-        <f>M16/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="N21" s="11">
+        <f>SUM(I21:M21)</f>
+        <v/>
+      </c>
+      <c r="O21" s="11">
+        <f>M21/$C$5</f>
+        <v/>
+      </c>
+      <c r="P21" s="12">
+        <f>O21*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q21" s="12">
+        <f>O21/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R21" s="12">
+        <f>O21*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S21" s="13">
+        <f>O21/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Абдуллина Аделина Линаровна</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D22" s="14" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E22" s="14" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F22" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G17" s="11" t="inlineStr">
+      <c r="G22" s="14" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H17" s="11" t="n">
+      <c r="H22" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="13" t="n">
+      <c r="I22" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="13" t="n">
+      <c r="J22" s="16" t="n">
         <v>129104.22</v>
       </c>
-      <c r="K17" s="13" t="n">
+      <c r="K22" s="16" t="n">
         <v>690632</v>
       </c>
-      <c r="L17" s="13" t="n">
+      <c r="L22" s="16" t="n">
         <v>1072320</v>
       </c>
-      <c r="M17" s="13" t="n">
+      <c r="M22" s="16" t="n">
         <v>755000</v>
       </c>
-      <c r="N17" s="14">
-        <f>SUM(I17:M17)</f>
-        <v/>
-      </c>
-      <c r="O17" s="15">
-        <f>M17/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="N22" s="17">
+        <f>SUM(I22:M22)</f>
+        <v/>
+      </c>
+      <c r="O22" s="17">
+        <f>M22/$C$5</f>
+        <v/>
+      </c>
+      <c r="P22" s="18">
+        <f>O22*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q22" s="18">
+        <f>O22/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R22" s="18">
+        <f>O22*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S22" s="19">
+        <f>O22/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Демакова Дарья</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>ТХ</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n">
+      <c r="H23" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I23" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="8" t="n">
+      <c r="J23" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="8" t="n">
+      <c r="K23" s="10" t="n">
         <v>582823.1800000001</v>
       </c>
-      <c r="L18" s="8" t="n">
+      <c r="L23" s="10" t="n">
         <v>1530724</v>
       </c>
-      <c r="M18" s="8" t="n">
+      <c r="M23" s="10" t="n">
         <v>1167329</v>
       </c>
-      <c r="N18" s="9">
-        <f>SUM(I18:M18)</f>
-        <v/>
-      </c>
-      <c r="O18" s="10">
-        <f>M18/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="n">
+      <c r="N23" s="11">
+        <f>SUM(I23:M23)</f>
+        <v/>
+      </c>
+      <c r="O23" s="11">
+        <f>M23/$C$5</f>
+        <v/>
+      </c>
+      <c r="P23" s="12">
+        <f>O23*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q23" s="12">
+        <f>O23/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R23" s="12">
+        <f>O23*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S23" s="13">
+        <f>O23/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>Возмищева Ксения Дмитриевна</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ОРБ)</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F24" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G19" s="11" t="inlineStr">
+      <c r="G24" s="14" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H19" s="11" t="n">
+      <c r="H24" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I19" s="13" t="n">
+      <c r="I24" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="13" t="n">
+      <c r="J24" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="13" t="n">
+      <c r="K24" s="16" t="n">
         <v>333311.66</v>
       </c>
-      <c r="L19" s="13" t="n">
+      <c r="L24" s="16" t="n">
         <v>1347175.74</v>
       </c>
-      <c r="M19" s="13" t="n">
+      <c r="M24" s="16" t="n">
         <v>1267879.25</v>
       </c>
-      <c r="N19" s="14">
-        <f>SUM(I19:M19)</f>
-        <v/>
-      </c>
-      <c r="O19" s="15">
-        <f>M19/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
+      <c r="N24" s="17">
+        <f>SUM(I24:M24)</f>
+        <v/>
+      </c>
+      <c r="O24" s="17">
+        <f>M24/$C$5</f>
+        <v/>
+      </c>
+      <c r="P24" s="18">
+        <f>O24*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q24" s="18">
+        <f>O24/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R24" s="18">
+        <f>O24*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S24" s="19">
+        <f>O24/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>Кузнецова Светлана Дмитриевна</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H20" s="6" t="n">
+      <c r="H25" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I25" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="J25" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="8" t="n">
+      <c r="K25" s="10" t="n">
         <v>1425506.19</v>
       </c>
-      <c r="L20" s="8" t="n">
+      <c r="L25" s="10" t="n">
         <v>109043</v>
       </c>
-      <c r="M20" s="8" t="n">
+      <c r="M25" s="10" t="n">
         <v>1145357.79</v>
       </c>
-      <c r="N20" s="9">
-        <f>SUM(I20:M20)</f>
-        <v/>
-      </c>
-      <c r="O20" s="10">
-        <f>M20/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="n">
+      <c r="N25" s="11">
+        <f>SUM(I25:M25)</f>
+        <v/>
+      </c>
+      <c r="O25" s="11">
+        <f>M25/$C$5</f>
+        <v/>
+      </c>
+      <c r="P25" s="12">
+        <f>O25*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q25" s="12">
+        <f>O25/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R25" s="12">
+        <f>O25*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S25" s="13">
+        <f>O25/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Нуруллина Анжелика Альбертовна</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D26" s="14" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E26" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
+      <c r="G26" s="14" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H21" s="11" t="n">
+      <c r="H26" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I21" s="13" t="n">
+      <c r="I26" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J21" s="13" t="n">
+      <c r="J26" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="K21" s="13" t="n">
+      <c r="K26" s="16" t="n">
         <v>338830</v>
       </c>
-      <c r="L21" s="13" t="n">
+      <c r="L26" s="16" t="n">
         <v>1331065</v>
       </c>
-      <c r="M21" s="13" t="n">
+      <c r="M26" s="16" t="n">
         <v>741701</v>
       </c>
-      <c r="N21" s="14">
-        <f>SUM(I21:M21)</f>
-        <v/>
-      </c>
-      <c r="O21" s="15">
-        <f>M21/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
+      <c r="N26" s="17">
+        <f>SUM(I26:M26)</f>
+        <v/>
+      </c>
+      <c r="O26" s="17">
+        <f>M26/$C$5</f>
+        <v/>
+      </c>
+      <c r="P26" s="18">
+        <f>O26*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q26" s="18">
+        <f>O26/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R26" s="18">
+        <f>O26*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S26" s="19">
+        <f>O26/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Тупико Олег Николаевич</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>ГК (общие)</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F27" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="H27" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="I22" s="8" t="n">
+      <c r="I27" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="8" t="n">
+      <c r="J27" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="8" t="n">
+      <c r="K27" s="10" t="n">
         <v>259907</v>
       </c>
-      <c r="L22" s="8" t="n">
+      <c r="L27" s="10" t="n">
         <v>337036</v>
       </c>
-      <c r="M22" s="8" t="n">
+      <c r="M27" s="10" t="n">
         <v>1219304</v>
       </c>
-      <c r="N22" s="9">
-        <f>SUM(I22:M22)</f>
-        <v/>
-      </c>
-      <c r="O22" s="10">
-        <f>M22/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="n">
+      <c r="N27" s="11">
+        <f>SUM(I27:M27)</f>
+        <v/>
+      </c>
+      <c r="O27" s="11">
+        <f>M27/$C$5</f>
+        <v/>
+      </c>
+      <c r="P27" s="12">
+        <f>O27*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q27" s="12">
+        <f>O27/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R27" s="12">
+        <f>O27*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S27" s="13">
+        <f>O27/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>Лукьянова Вера Константиновна</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
+      <c r="D28" s="14" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E23" s="11" t="inlineStr">
+      <c r="E28" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F23" s="11" t="inlineStr">
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G23" s="11" t="inlineStr">
+      <c r="G28" s="14" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H23" s="11" t="n">
+      <c r="H28" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I23" s="13" t="n">
+      <c r="I28" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J23" s="13" t="n">
+      <c r="J28" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="13" t="n">
+      <c r="K28" s="16" t="n">
         <v>141702</v>
       </c>
-      <c r="L23" s="13" t="n">
+      <c r="L28" s="16" t="n">
         <v>73617</v>
       </c>
-      <c r="M23" s="13" t="n">
+      <c r="M28" s="16" t="n">
         <v>973404</v>
       </c>
-      <c r="N23" s="14">
-        <f>SUM(I23:M23)</f>
-        <v/>
-      </c>
-      <c r="O23" s="15">
-        <f>M23/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="N28" s="17">
+        <f>SUM(I28:M28)</f>
+        <v/>
+      </c>
+      <c r="O28" s="17">
+        <f>M28/$C$5</f>
+        <v/>
+      </c>
+      <c r="P28" s="18">
+        <f>O28*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q28" s="18">
+        <f>O28/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R28" s="18">
+        <f>O28*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S28" s="19">
+        <f>O28/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Левашева Анна Алексеевна</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D29" s="8" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>2025–2026</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n">
+      <c r="H29" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="I24" s="8" t="n">
+      <c r="I29" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="8" t="n">
+      <c r="J29" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="8" t="n">
+      <c r="K29" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="8" t="n">
+      <c r="L29" s="10" t="n">
         <v>798831.01</v>
       </c>
-      <c r="M24" s="8" t="n">
+      <c r="M29" s="10" t="n">
         <v>1362100.09</v>
       </c>
-      <c r="N24" s="9">
-        <f>SUM(I24:M24)</f>
-        <v/>
-      </c>
-      <c r="O24" s="10">
-        <f>M24/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="N29" s="11">
+        <f>SUM(I29:M29)</f>
+        <v/>
+      </c>
+      <c r="O29" s="11">
+        <f>M29/$C$5</f>
+        <v/>
+      </c>
+      <c r="P29" s="12">
+        <f>O29*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q29" s="12">
+        <f>O29/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R29" s="12">
+        <f>O29*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S29" s="13">
+        <f>O29/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>Капустина Вероника Сергеевна</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>ТФМ (ОСК)</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F30" s="14" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G25" s="11" t="inlineStr">
+      <c r="G30" s="14" t="inlineStr">
         <is>
           <t>2025–2026</t>
         </is>
       </c>
-      <c r="H25" s="11" t="n">
+      <c r="H30" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="I25" s="13" t="n">
+      <c r="I30" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="13" t="n">
+      <c r="J30" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="13" t="n">
+      <c r="K30" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L25" s="13" t="n">
+      <c r="L30" s="16" t="n">
         <v>214440.3</v>
       </c>
-      <c r="M25" s="13" t="n">
+      <c r="M30" s="16" t="n">
         <v>1228052.73</v>
       </c>
-      <c r="N25" s="14">
-        <f>SUM(I25:M25)</f>
-        <v/>
-      </c>
-      <c r="O25" s="15">
-        <f>M25/$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="16" t="inlineStr"/>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="N30" s="17">
+        <f>SUM(I30:M30)</f>
+        <v/>
+      </c>
+      <c r="O30" s="17">
+        <f>M30/$C$5</f>
+        <v/>
+      </c>
+      <c r="P30" s="18">
+        <f>O30*$C$6</f>
+        <v/>
+      </c>
+      <c r="Q30" s="18">
+        <f>O30/(1-$C$7)</f>
+        <v/>
+      </c>
+      <c r="R30" s="18">
+        <f>O30*(1+$C$8)</f>
+        <v/>
+      </c>
+      <c r="S30" s="19">
+        <f>O30/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="n"/>
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>ИТОГО (20 чел.)</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n"/>
-      <c r="D26" s="16" t="n"/>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="16" t="n"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
-      <c r="I26" s="18">
-        <f>SUM(I6:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="18">
-        <f>SUM(J6:J25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="18">
-        <f>SUM(K6:K25)</f>
-        <v/>
-      </c>
-      <c r="L26" s="18">
-        <f>SUM(L6:L25)</f>
-        <v/>
-      </c>
-      <c r="M26" s="18">
-        <f>SUM(M6:M25)</f>
-        <v/>
-      </c>
-      <c r="N26" s="18">
-        <f>SUM(N6:N25)</f>
-        <v/>
-      </c>
-      <c r="O26" s="18">
-        <f>SUM(O6:O25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="20" t="n"/>
+      <c r="E31" s="20" t="n"/>
+      <c r="F31" s="20" t="n"/>
+      <c r="G31" s="20" t="n"/>
+      <c r="H31" s="20" t="n"/>
+      <c r="I31" s="22">
+        <f>SUM(I11:I30)</f>
+        <v/>
+      </c>
+      <c r="J31" s="22">
+        <f>SUM(J11:J30)</f>
+        <v/>
+      </c>
+      <c r="K31" s="22">
+        <f>SUM(K11:K30)</f>
+        <v/>
+      </c>
+      <c r="L31" s="22">
+        <f>SUM(L11:L30)</f>
+        <v/>
+      </c>
+      <c r="M31" s="22">
+        <f>SUM(M11:M30)</f>
+        <v/>
+      </c>
+      <c r="N31" s="22">
+        <f>SUM(N11:N30)</f>
+        <v/>
+      </c>
+      <c r="O31" s="22">
+        <f>SUM(O11:O30)</f>
+        <v/>
+      </c>
+      <c r="P31" s="22">
+        <f>SUM(P11:P30)</f>
+        <v/>
+      </c>
+      <c r="Q31" s="22">
+        <f>SUM(Q11:Q30)</f>
+        <v/>
+      </c>
+      <c r="R31" s="22">
+        <f>SUM(R11:R30)</f>
+        <v/>
+      </c>
+      <c r="S31" s="22">
+        <f>SUM(S11:S30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>ПЛАНИРОВАНИЕ</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="24" t="inlineStr">
+        <is>
+          <t>Месячный фонд (итого к оплате)</t>
+        </is>
+      </c>
+      <c r="B34" s="25" t="inlineStr"/>
+      <c r="C34" s="26">
+        <f>S31*1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>На 6 месяцев</t>
+        </is>
+      </c>
+      <c r="B35" s="25" t="inlineStr"/>
+      <c r="C35" s="26">
+        <f>S31*6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
+        <is>
+          <t>На 12 месяцев</t>
+        </is>
+      </c>
+      <c r="B36" s="25" t="inlineStr"/>
+      <c r="C36" s="26">
+        <f>S31*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="27" t="inlineStr">
         <is>
           <t>Примечания</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>1. Данные получены через Google Drive API. Годовые итоги взяты из сводных таблиц листов; помесячные строки в выгрузке неполные.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>2. Устранено задвоение строк между листами-копиями («2023 (копия)», параллельные вкладки 2025).</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>3. Столбец «Лет» — число календарных лет, в которых были выплаты. «Период выплат» — первый и последний год с выплатами.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>4. Левашева и Капустина получают выплаты 2 года (2025–2026) — под критерий «более 2 лет» не подходят, включены по отдельной просьбе.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>5. Левашева — смена фамилии с 23.09.25 (Домрачева); данные до смены могут учитываться отдельно.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>6. Ставка НПД 0% — выплаты без налога на профдоход (по данным справочника СЗ).</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>7. Среднемесячная выплата 2026 = «Итого 2026» ÷ 7 (число выплат в 2026 г., январь–июль). Это фактический месячный run-rate по начислениям декабрь 2025 – июнь 2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>8. Ограничение выгрузки: по фамилиям после ~«Л» ранние годы (2022–2024) могли не попасть в сводные — стаж и суммы у них могут быть занижены.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="19" t="inlineStr">
-        <is>
-          <t>ПЛАНИРОВАНИЕ</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>Плановый месячный фонд (сумма среднемесячных выплат)</t>
-        </is>
-      </c>
-      <c r="B39" s="21" t="inlineStr"/>
-      <c r="C39" s="22">
-        <f>O26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="20" t="inlineStr">
-        <is>
-          <t>На 6 месяцев</t>
-        </is>
-      </c>
-      <c r="B40" s="21" t="inlineStr"/>
-      <c r="C40" s="22">
-        <f>O26*6</f>
-        <v/>
-      </c>
-    </row>
     <row r="41">
-      <c r="A41" s="20" t="inlineStr">
-        <is>
-          <t>На 12 месяцев</t>
-        </is>
-      </c>
-      <c r="B41" s="21" t="inlineStr"/>
-      <c r="C41" s="22">
-        <f>O26*12</f>
-        <v/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>3. «Лет» — число календарных лет с выплатами. «Период выплат» — первый и последний год с выплатами.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>4. Среднемесячная выплата 2026 = «Итого 2026» ÷ C5. Это фактический месячный run-rate по начислениям декабрь 2025 – июнь 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>5. ВАЖНО: базовая сумма — «Итого к выплате», она УЖЕ включает НПД. Столбец «С НПД +6%» начисляет налог поверх этой суммы. Если нужен НПД на сумму «на руки», базу надо заменить.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>6. «ИТОГО к оплате в месяц» = среднемесячная ÷ 0,975 × 1,06 × 1,03 (сбор ЮЛ Сингапура → НПД → комиссия 4dev).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>7. Левашева и Капустина получают выплаты 2 года (2025–2026) — под критерий «более 2 лет» не подходят, включены по отдельной просьбе.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>8. Левашева — смена фамилии с 23.09.25 (Домрачева). Ставка НПД 0% в справочнике — выплаты без налога на профдоход.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>9. Ограничение выгрузки: по фамилиям после ~«Л» ранние годы (2022–2024) могли не попасть в сводные — стаж и суммы у них могут быть занижены.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O25"/>
+  <autoFilter ref="A10:S30"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Show Singapore fee and NPD as amounts, not grossed-up totals
Columns Q and R now carry the 2.5% Singapore entity fee and the 6% NPD
as rouble amounts, matching how the 4dev commission column already read.
The monthly total becomes a plain sum of base plus the three add-ons
instead of a compounding chain.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wo4Lmevz8VeqLa4QdqkBF
</commit_message>
<xml_diff>
--- a/СЗ_длительные_выплаты_2022-2026.xlsx
+++ b/СЗ_длительные_выплаты_2022-2026.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S47"/>
+  <dimension ref="A1:S48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -747,12 +747,12 @@
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>Со сбором ЮЛ Сингапур (÷0,975)</t>
+          <t>Сбор ЮЛ Сингапура 2,5%</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
         <is>
-          <t>С НПД +6%</t>
+          <t>НПД 6%</t>
         </is>
       </c>
       <c r="S10" s="7" t="inlineStr">
@@ -826,15 +826,15 @@
         <v/>
       </c>
       <c r="Q11" s="12">
-        <f>O11/(1-$C$7)</f>
+        <f>O11/(1-$C$7)-O11</f>
         <v/>
       </c>
       <c r="R11" s="12">
-        <f>O11*(1+$C$8)</f>
+        <f>O11*$C$8</f>
         <v/>
       </c>
       <c r="S11" s="13">
-        <f>O11/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O11+P11+Q11+R11</f>
         <v/>
       </c>
     </row>
@@ -903,15 +903,15 @@
         <v/>
       </c>
       <c r="Q12" s="18">
-        <f>O12/(1-$C$7)</f>
+        <f>O12/(1-$C$7)-O12</f>
         <v/>
       </c>
       <c r="R12" s="18">
-        <f>O12*(1+$C$8)</f>
+        <f>O12*$C$8</f>
         <v/>
       </c>
       <c r="S12" s="19">
-        <f>O12/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O12+P12+Q12+R12</f>
         <v/>
       </c>
     </row>
@@ -980,15 +980,15 @@
         <v/>
       </c>
       <c r="Q13" s="12">
-        <f>O13/(1-$C$7)</f>
+        <f>O13/(1-$C$7)-O13</f>
         <v/>
       </c>
       <c r="R13" s="12">
-        <f>O13*(1+$C$8)</f>
+        <f>O13*$C$8</f>
         <v/>
       </c>
       <c r="S13" s="13">
-        <f>O13/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O13+P13+Q13+R13</f>
         <v/>
       </c>
     </row>
@@ -1057,15 +1057,15 @@
         <v/>
       </c>
       <c r="Q14" s="18">
-        <f>O14/(1-$C$7)</f>
+        <f>O14/(1-$C$7)-O14</f>
         <v/>
       </c>
       <c r="R14" s="18">
-        <f>O14*(1+$C$8)</f>
+        <f>O14*$C$8</f>
         <v/>
       </c>
       <c r="S14" s="19">
-        <f>O14/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O14+P14+Q14+R14</f>
         <v/>
       </c>
     </row>
@@ -1134,15 +1134,15 @@
         <v/>
       </c>
       <c r="Q15" s="12">
-        <f>O15/(1-$C$7)</f>
+        <f>O15/(1-$C$7)-O15</f>
         <v/>
       </c>
       <c r="R15" s="12">
-        <f>O15*(1+$C$8)</f>
+        <f>O15*$C$8</f>
         <v/>
       </c>
       <c r="S15" s="13">
-        <f>O15/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O15+P15+Q15+R15</f>
         <v/>
       </c>
     </row>
@@ -1211,15 +1211,15 @@
         <v/>
       </c>
       <c r="Q16" s="18">
-        <f>O16/(1-$C$7)</f>
+        <f>O16/(1-$C$7)-O16</f>
         <v/>
       </c>
       <c r="R16" s="18">
-        <f>O16*(1+$C$8)</f>
+        <f>O16*$C$8</f>
         <v/>
       </c>
       <c r="S16" s="19">
-        <f>O16/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O16+P16+Q16+R16</f>
         <v/>
       </c>
     </row>
@@ -1288,15 +1288,15 @@
         <v/>
       </c>
       <c r="Q17" s="12">
-        <f>O17/(1-$C$7)</f>
+        <f>O17/(1-$C$7)-O17</f>
         <v/>
       </c>
       <c r="R17" s="12">
-        <f>O17*(1+$C$8)</f>
+        <f>O17*$C$8</f>
         <v/>
       </c>
       <c r="S17" s="13">
-        <f>O17/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O17+P17+Q17+R17</f>
         <v/>
       </c>
     </row>
@@ -1365,15 +1365,15 @@
         <v/>
       </c>
       <c r="Q18" s="18">
-        <f>O18/(1-$C$7)</f>
+        <f>O18/(1-$C$7)-O18</f>
         <v/>
       </c>
       <c r="R18" s="18">
-        <f>O18*(1+$C$8)</f>
+        <f>O18*$C$8</f>
         <v/>
       </c>
       <c r="S18" s="19">
-        <f>O18/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O18+P18+Q18+R18</f>
         <v/>
       </c>
     </row>
@@ -1442,15 +1442,15 @@
         <v/>
       </c>
       <c r="Q19" s="12">
-        <f>O19/(1-$C$7)</f>
+        <f>O19/(1-$C$7)-O19</f>
         <v/>
       </c>
       <c r="R19" s="12">
-        <f>O19*(1+$C$8)</f>
+        <f>O19*$C$8</f>
         <v/>
       </c>
       <c r="S19" s="13">
-        <f>O19/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O19+P19+Q19+R19</f>
         <v/>
       </c>
     </row>
@@ -1519,15 +1519,15 @@
         <v/>
       </c>
       <c r="Q20" s="18">
-        <f>O20/(1-$C$7)</f>
+        <f>O20/(1-$C$7)-O20</f>
         <v/>
       </c>
       <c r="R20" s="18">
-        <f>O20*(1+$C$8)</f>
+        <f>O20*$C$8</f>
         <v/>
       </c>
       <c r="S20" s="19">
-        <f>O20/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O20+P20+Q20+R20</f>
         <v/>
       </c>
     </row>
@@ -1596,15 +1596,15 @@
         <v/>
       </c>
       <c r="Q21" s="12">
-        <f>O21/(1-$C$7)</f>
+        <f>O21/(1-$C$7)-O21</f>
         <v/>
       </c>
       <c r="R21" s="12">
-        <f>O21*(1+$C$8)</f>
+        <f>O21*$C$8</f>
         <v/>
       </c>
       <c r="S21" s="13">
-        <f>O21/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O21+P21+Q21+R21</f>
         <v/>
       </c>
     </row>
@@ -1673,15 +1673,15 @@
         <v/>
       </c>
       <c r="Q22" s="18">
-        <f>O22/(1-$C$7)</f>
+        <f>O22/(1-$C$7)-O22</f>
         <v/>
       </c>
       <c r="R22" s="18">
-        <f>O22*(1+$C$8)</f>
+        <f>O22*$C$8</f>
         <v/>
       </c>
       <c r="S22" s="19">
-        <f>O22/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O22+P22+Q22+R22</f>
         <v/>
       </c>
     </row>
@@ -1750,15 +1750,15 @@
         <v/>
       </c>
       <c r="Q23" s="12">
-        <f>O23/(1-$C$7)</f>
+        <f>O23/(1-$C$7)-O23</f>
         <v/>
       </c>
       <c r="R23" s="12">
-        <f>O23*(1+$C$8)</f>
+        <f>O23*$C$8</f>
         <v/>
       </c>
       <c r="S23" s="13">
-        <f>O23/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O23+P23+Q23+R23</f>
         <v/>
       </c>
     </row>
@@ -1827,15 +1827,15 @@
         <v/>
       </c>
       <c r="Q24" s="18">
-        <f>O24/(1-$C$7)</f>
+        <f>O24/(1-$C$7)-O24</f>
         <v/>
       </c>
       <c r="R24" s="18">
-        <f>O24*(1+$C$8)</f>
+        <f>O24*$C$8</f>
         <v/>
       </c>
       <c r="S24" s="19">
-        <f>O24/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O24+P24+Q24+R24</f>
         <v/>
       </c>
     </row>
@@ -1904,15 +1904,15 @@
         <v/>
       </c>
       <c r="Q25" s="12">
-        <f>O25/(1-$C$7)</f>
+        <f>O25/(1-$C$7)-O25</f>
         <v/>
       </c>
       <c r="R25" s="12">
-        <f>O25*(1+$C$8)</f>
+        <f>O25*$C$8</f>
         <v/>
       </c>
       <c r="S25" s="13">
-        <f>O25/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O25+P25+Q25+R25</f>
         <v/>
       </c>
     </row>
@@ -1981,15 +1981,15 @@
         <v/>
       </c>
       <c r="Q26" s="18">
-        <f>O26/(1-$C$7)</f>
+        <f>O26/(1-$C$7)-O26</f>
         <v/>
       </c>
       <c r="R26" s="18">
-        <f>O26*(1+$C$8)</f>
+        <f>O26*$C$8</f>
         <v/>
       </c>
       <c r="S26" s="19">
-        <f>O26/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O26+P26+Q26+R26</f>
         <v/>
       </c>
     </row>
@@ -2058,15 +2058,15 @@
         <v/>
       </c>
       <c r="Q27" s="12">
-        <f>O27/(1-$C$7)</f>
+        <f>O27/(1-$C$7)-O27</f>
         <v/>
       </c>
       <c r="R27" s="12">
-        <f>O27*(1+$C$8)</f>
+        <f>O27*$C$8</f>
         <v/>
       </c>
       <c r="S27" s="13">
-        <f>O27/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O27+P27+Q27+R27</f>
         <v/>
       </c>
     </row>
@@ -2135,15 +2135,15 @@
         <v/>
       </c>
       <c r="Q28" s="18">
-        <f>O28/(1-$C$7)</f>
+        <f>O28/(1-$C$7)-O28</f>
         <v/>
       </c>
       <c r="R28" s="18">
-        <f>O28*(1+$C$8)</f>
+        <f>O28*$C$8</f>
         <v/>
       </c>
       <c r="S28" s="19">
-        <f>O28/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O28+P28+Q28+R28</f>
         <v/>
       </c>
     </row>
@@ -2212,15 +2212,15 @@
         <v/>
       </c>
       <c r="Q29" s="12">
-        <f>O29/(1-$C$7)</f>
+        <f>O29/(1-$C$7)-O29</f>
         <v/>
       </c>
       <c r="R29" s="12">
-        <f>O29*(1+$C$8)</f>
+        <f>O29*$C$8</f>
         <v/>
       </c>
       <c r="S29" s="13">
-        <f>O29/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O29+P29+Q29+R29</f>
         <v/>
       </c>
     </row>
@@ -2289,15 +2289,15 @@
         <v/>
       </c>
       <c r="Q30" s="18">
-        <f>O30/(1-$C$7)</f>
+        <f>O30/(1-$C$7)-O30</f>
         <v/>
       </c>
       <c r="R30" s="18">
-        <f>O30*(1+$C$8)</f>
+        <f>O30*$C$8</f>
         <v/>
       </c>
       <c r="S30" s="19">
-        <f>O30/(1-$C$7)*(1+$C$8)*(1+$C$6)</f>
+        <f>O30+P30+Q30+R30</f>
         <v/>
       </c>
     </row>
@@ -2447,28 +2447,35 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>6. «ИТОГО к оплате в месяц» = среднемесячная ÷ 0,975 × 1,06 × 1,03 (сбор ЮЛ Сингапура → НПД → комиссия 4dev).</t>
+          <t>6. Все три надбавки считаются от среднемесячной выплаты: комиссия 4dev = ×3%; сбор ЮЛ Сингапура = ÷0,975 − среднемесячная (2,5% сверху); НПД = ×6%.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>7. Левашева и Капустина получают выплаты 2 года (2025–2026) — под критерий «более 2 лет» не подходят, включены по отдельной просьбе.</t>
+          <t>7. «ИТОГО к оплате в месяц» = среднемесячная + комиссия + сбор + НПД (надбавки не каскадируются). Если применять их последовательно (÷0,975 × 1,06 × 1,03), итог по группе будет 3 830 014 ₽ вместо 3 815 806 ₽.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>8. Левашева — смена фамилии с 23.09.25 (Домрачева). Ставка НПД 0% в справочнике — выплаты без налога на профдоход.</t>
+          <t>8. Левашева и Капустина получают выплаты 2 года (2025–2026) — под критерий «более 2 лет» не подходят, включены по отдельной просьбе.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>9. Ограничение выгрузки: по фамилиям после ~«Л» ранние годы (2022–2024) могли не попасть в сводные — стаж и суммы у них могут быть занижены.</t>
+          <t>9. Левашева — смена фамилии с 23.09.25 (Домрачева). Ставка НПД 0% в справочнике — выплаты без налога на профдоход.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>10. Ограничение выгрузки: по фамилиям после ~«Л» ранние годы (2022–2024) могли не попасть в сводные — стаж и суммы у них могут быть занижены.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebase monthly cost columns on net pay instead of gross
The 2026 run-rate now converts to net ("na ruki") by multiplying the
gross by (1 - NPD rate), which mirrors how the source sheet derives
gross from net. Each person's own NPD rate lives in a hidden column, so
the zero-rate case is handled instead of assuming 6% for everyone, and
the tax add-on reconstructs the original gross exactly.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019wo4Lmevz8VeqLa4QdqkBF
</commit_message>
<xml_diff>
--- a/СЗ_длительные_выплаты_2022-2026.xlsx
+++ b/СЗ_длительные_выплаты_2022-2026.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0;(#,##0);-"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -148,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,25 +173,26 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -552,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S48"/>
+  <dimension ref="A1:T48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -574,6 +580,7 @@
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="20" customWidth="1" min="19" max="19"/>
+    <col hidden="1" width="13" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -652,7 +659,7 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Ставка НПД</t>
+          <t>Ставка НПД (базовая)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
@@ -660,7 +667,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>← начисляется сверху на среднемесячную</t>
+          <t>← фактическая ставка по каждому — в скрытом столбце T</t>
         </is>
       </c>
     </row>
@@ -737,7 +744,7 @@
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
-          <t>Среднемес. выплата 2026</t>
+          <t>Среднемес. на руки 2026</t>
         </is>
       </c>
       <c r="P10" s="7" t="inlineStr">
@@ -818,7 +825,7 @@
         <v/>
       </c>
       <c r="O11" s="11">
-        <f>M11/$C$5</f>
+        <f>M11/$C$5*(1-T11)</f>
         <v/>
       </c>
       <c r="P11" s="12">
@@ -830,89 +837,95 @@
         <v/>
       </c>
       <c r="R11" s="12">
-        <f>O11*$C$8</f>
+        <f>IF(T11=0,0,O11/(1-T11)-O11)</f>
         <v/>
       </c>
       <c r="S11" s="13">
         <f>O11+P11+Q11+R11</f>
         <v/>
       </c>
+      <c r="T11" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="n">
+      <c r="A12" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>Высочинский Даниил Сергеевич</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ОСП)</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H12" s="14" t="n">
+      <c r="H12" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="I12" s="16" t="n">
+      <c r="I12" s="17" t="n">
         <v>43489</v>
       </c>
-      <c r="J12" s="16" t="n">
+      <c r="J12" s="17" t="n">
         <v>715306.13</v>
       </c>
-      <c r="K12" s="16" t="n">
+      <c r="K12" s="17" t="n">
         <v>1582317</v>
       </c>
-      <c r="L12" s="16" t="n">
+      <c r="L12" s="17" t="n">
         <v>1778297</v>
       </c>
-      <c r="M12" s="16" t="n">
+      <c r="M12" s="17" t="n">
         <v>1146293</v>
       </c>
-      <c r="N12" s="17">
+      <c r="N12" s="18">
         <f>SUM(I12:M12)</f>
         <v/>
       </c>
-      <c r="O12" s="17">
-        <f>M12/$C$5</f>
-        <v/>
-      </c>
-      <c r="P12" s="18">
+      <c r="O12" s="18">
+        <f>M12/$C$5*(1-T12)</f>
+        <v/>
+      </c>
+      <c r="P12" s="19">
         <f>O12*$C$6</f>
         <v/>
       </c>
-      <c r="Q12" s="18">
+      <c r="Q12" s="19">
         <f>O12/(1-$C$7)-O12</f>
         <v/>
       </c>
-      <c r="R12" s="18">
-        <f>O12*$C$8</f>
-        <v/>
-      </c>
-      <c r="S12" s="19">
+      <c r="R12" s="19">
+        <f>IF(T12=0,0,O12/(1-T12)-O12)</f>
+        <v/>
+      </c>
+      <c r="S12" s="20">
         <f>O12+P12+Q12+R12</f>
         <v/>
+      </c>
+      <c r="T12" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="13">
@@ -972,7 +985,7 @@
         <v/>
       </c>
       <c r="O13" s="11">
-        <f>M13/$C$5</f>
+        <f>M13/$C$5*(1-T13)</f>
         <v/>
       </c>
       <c r="P13" s="12">
@@ -984,89 +997,95 @@
         <v/>
       </c>
       <c r="R13" s="12">
-        <f>O13*$C$8</f>
+        <f>IF(T13=0,0,O13/(1-T13)-O13)</f>
         <v/>
       </c>
       <c r="S13" s="13">
         <f>O13+P13+Q13+R13</f>
         <v/>
       </c>
+      <c r="T13" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="n">
+      <c r="A14" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Грудинин Алексей Сергеевич</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F14" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H14" s="14" t="n">
+      <c r="H14" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="16" t="n">
+      <c r="I14" s="17" t="n">
         <v>267577.88</v>
       </c>
-      <c r="J14" s="16" t="n">
+      <c r="J14" s="17" t="n">
         <v>960405.97</v>
       </c>
-      <c r="K14" s="16" t="n">
+      <c r="K14" s="17" t="n">
         <v>1372957.36</v>
       </c>
-      <c r="L14" s="16" t="n">
+      <c r="L14" s="17" t="n">
         <v>1558585.08</v>
       </c>
-      <c r="M14" s="16" t="n">
+      <c r="M14" s="17" t="n">
         <v>938053.12</v>
       </c>
-      <c r="N14" s="17">
+      <c r="N14" s="18">
         <f>SUM(I14:M14)</f>
         <v/>
       </c>
-      <c r="O14" s="17">
-        <f>M14/$C$5</f>
-        <v/>
-      </c>
-      <c r="P14" s="18">
+      <c r="O14" s="18">
+        <f>M14/$C$5*(1-T14)</f>
+        <v/>
+      </c>
+      <c r="P14" s="19">
         <f>O14*$C$6</f>
         <v/>
       </c>
-      <c r="Q14" s="18">
+      <c r="Q14" s="19">
         <f>O14/(1-$C$7)-O14</f>
         <v/>
       </c>
-      <c r="R14" s="18">
-        <f>O14*$C$8</f>
-        <v/>
-      </c>
-      <c r="S14" s="19">
+      <c r="R14" s="19">
+        <f>IF(T14=0,0,O14/(1-T14)-O14)</f>
+        <v/>
+      </c>
+      <c r="S14" s="20">
         <f>O14+P14+Q14+R14</f>
         <v/>
+      </c>
+      <c r="T14" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="15">
@@ -1126,7 +1145,7 @@
         <v/>
       </c>
       <c r="O15" s="11">
-        <f>M15/$C$5</f>
+        <f>M15/$C$5*(1-T15)</f>
         <v/>
       </c>
       <c r="P15" s="12">
@@ -1138,89 +1157,95 @@
         <v/>
       </c>
       <c r="R15" s="12">
-        <f>O15*$C$8</f>
+        <f>IF(T15=0,0,O15/(1-T15)-O15)</f>
         <v/>
       </c>
       <c r="S15" s="13">
         <f>O15+P15+Q15+R15</f>
         <v/>
       </c>
+      <c r="T15" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="n">
+      <c r="A16" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Репетенко Инна Эдуардовна</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ОРБ)</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
         <is>
           <t>2022–2026</t>
         </is>
       </c>
-      <c r="H16" s="14" t="n">
+      <c r="H16" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="I16" s="16" t="n">
+      <c r="I16" s="17" t="n">
         <v>112190</v>
       </c>
-      <c r="J16" s="16" t="n">
+      <c r="J16" s="17" t="n">
         <v>246600</v>
       </c>
-      <c r="K16" s="16" t="n">
+      <c r="K16" s="17" t="n">
         <v>415655.93</v>
       </c>
-      <c r="L16" s="16" t="n">
+      <c r="L16" s="17" t="n">
         <v>142973.52</v>
       </c>
-      <c r="M16" s="16" t="n">
+      <c r="M16" s="17" t="n">
         <v>905821.35</v>
       </c>
-      <c r="N16" s="17">
+      <c r="N16" s="18">
         <f>SUM(I16:M16)</f>
         <v/>
       </c>
-      <c r="O16" s="17">
-        <f>M16/$C$5</f>
-        <v/>
-      </c>
-      <c r="P16" s="18">
+      <c r="O16" s="18">
+        <f>M16/$C$5*(1-T16)</f>
+        <v/>
+      </c>
+      <c r="P16" s="19">
         <f>O16*$C$6</f>
         <v/>
       </c>
-      <c r="Q16" s="18">
+      <c r="Q16" s="19">
         <f>O16/(1-$C$7)-O16</f>
         <v/>
       </c>
-      <c r="R16" s="18">
-        <f>O16*$C$8</f>
-        <v/>
-      </c>
-      <c r="S16" s="19">
+      <c r="R16" s="19">
+        <f>IF(T16=0,0,O16/(1-T16)-O16)</f>
+        <v/>
+      </c>
+      <c r="S16" s="20">
         <f>O16+P16+Q16+R16</f>
         <v/>
+      </c>
+      <c r="T16" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="17">
@@ -1280,7 +1305,7 @@
         <v/>
       </c>
       <c r="O17" s="11">
-        <f>M17/$C$5</f>
+        <f>M17/$C$5*(1-T17)</f>
         <v/>
       </c>
       <c r="P17" s="12">
@@ -1292,89 +1317,95 @@
         <v/>
       </c>
       <c r="R17" s="12">
-        <f>O17*$C$8</f>
+        <f>IF(T17=0,0,O17/(1-T17)-O17)</f>
         <v/>
       </c>
       <c r="S17" s="13">
         <f>O17+P17+Q17+R17</f>
         <v/>
       </c>
+      <c r="T17" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="n">
+      <c r="A18" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Жиркова Валентина Александровна</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="G18" s="15" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H18" s="14" t="n">
+      <c r="H18" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="I18" s="16" t="n">
+      <c r="I18" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J18" s="16" t="n">
+      <c r="J18" s="17" t="n">
         <v>257222.24</v>
       </c>
-      <c r="K18" s="16" t="n">
+      <c r="K18" s="17" t="n">
         <v>1497661</v>
       </c>
-      <c r="L18" s="16" t="n">
+      <c r="L18" s="17" t="n">
         <v>2201639.5</v>
       </c>
-      <c r="M18" s="16" t="n">
+      <c r="M18" s="17" t="n">
         <v>1656517.19</v>
       </c>
-      <c r="N18" s="17">
+      <c r="N18" s="18">
         <f>SUM(I18:M18)</f>
         <v/>
       </c>
-      <c r="O18" s="17">
-        <f>M18/$C$5</f>
-        <v/>
-      </c>
-      <c r="P18" s="18">
+      <c r="O18" s="18">
+        <f>M18/$C$5*(1-T18)</f>
+        <v/>
+      </c>
+      <c r="P18" s="19">
         <f>O18*$C$6</f>
         <v/>
       </c>
-      <c r="Q18" s="18">
+      <c r="Q18" s="19">
         <f>O18/(1-$C$7)-O18</f>
         <v/>
       </c>
-      <c r="R18" s="18">
-        <f>O18*$C$8</f>
-        <v/>
-      </c>
-      <c r="S18" s="19">
+      <c r="R18" s="19">
+        <f>IF(T18=0,0,O18/(1-T18)-O18)</f>
+        <v/>
+      </c>
+      <c r="S18" s="20">
         <f>O18+P18+Q18+R18</f>
         <v/>
+      </c>
+      <c r="T18" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="19">
@@ -1434,7 +1465,7 @@
         <v/>
       </c>
       <c r="O19" s="11">
-        <f>M19/$C$5</f>
+        <f>M19/$C$5*(1-T19)</f>
         <v/>
       </c>
       <c r="P19" s="12">
@@ -1446,89 +1477,95 @@
         <v/>
       </c>
       <c r="R19" s="12">
-        <f>O19*$C$8</f>
+        <f>IF(T19=0,0,O19/(1-T19)-O19)</f>
         <v/>
       </c>
       <c r="S19" s="13">
         <f>O19+P19+Q19+R19</f>
         <v/>
       </c>
+      <c r="T19" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="n">
+      <c r="A20" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Оглезнева Полина Сергеевна</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ОСП)</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G20" s="14" t="inlineStr">
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H20" s="14" t="n">
+      <c r="H20" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="I20" s="16" t="n">
+      <c r="I20" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J20" s="16" t="n">
+      <c r="J20" s="17" t="n">
         <v>140852</v>
       </c>
-      <c r="K20" s="16" t="n">
+      <c r="K20" s="17" t="n">
         <v>205851</v>
       </c>
-      <c r="L20" s="16" t="n">
+      <c r="L20" s="17" t="n">
         <v>2326991</v>
       </c>
-      <c r="M20" s="16" t="n">
+      <c r="M20" s="17" t="n">
         <v>1574518</v>
       </c>
-      <c r="N20" s="17">
+      <c r="N20" s="18">
         <f>SUM(I20:M20)</f>
         <v/>
       </c>
-      <c r="O20" s="17">
-        <f>M20/$C$5</f>
-        <v/>
-      </c>
-      <c r="P20" s="18">
+      <c r="O20" s="18">
+        <f>M20/$C$5*(1-T20)</f>
+        <v/>
+      </c>
+      <c r="P20" s="19">
         <f>O20*$C$6</f>
         <v/>
       </c>
-      <c r="Q20" s="18">
+      <c r="Q20" s="19">
         <f>O20/(1-$C$7)-O20</f>
         <v/>
       </c>
-      <c r="R20" s="18">
-        <f>O20*$C$8</f>
-        <v/>
-      </c>
-      <c r="S20" s="19">
+      <c r="R20" s="19">
+        <f>IF(T20=0,0,O20/(1-T20)-O20)</f>
+        <v/>
+      </c>
+      <c r="S20" s="20">
         <f>O20+P20+Q20+R20</f>
         <v/>
+      </c>
+      <c r="T20" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="21">
@@ -1588,7 +1625,7 @@
         <v/>
       </c>
       <c r="O21" s="11">
-        <f>M21/$C$5</f>
+        <f>M21/$C$5*(1-T21)</f>
         <v/>
       </c>
       <c r="P21" s="12">
@@ -1600,89 +1637,95 @@
         <v/>
       </c>
       <c r="R21" s="12">
-        <f>O21*$C$8</f>
+        <f>IF(T21=0,0,O21/(1-T21)-O21)</f>
         <v/>
       </c>
       <c r="S21" s="13">
         <f>O21+P21+Q21+R21</f>
         <v/>
       </c>
+      <c r="T21" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="n">
+      <c r="A22" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Абдуллина Аделина Линаровна</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>0%</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
+      <c r="G22" s="15" t="inlineStr">
         <is>
           <t>2023–2026</t>
         </is>
       </c>
-      <c r="H22" s="14" t="n">
+      <c r="H22" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="I22" s="16" t="n">
+      <c r="I22" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="16" t="n">
+      <c r="J22" s="17" t="n">
         <v>129104.22</v>
       </c>
-      <c r="K22" s="16" t="n">
+      <c r="K22" s="17" t="n">
         <v>690632</v>
       </c>
-      <c r="L22" s="16" t="n">
+      <c r="L22" s="17" t="n">
         <v>1072320</v>
       </c>
-      <c r="M22" s="16" t="n">
+      <c r="M22" s="17" t="n">
         <v>755000</v>
       </c>
-      <c r="N22" s="17">
+      <c r="N22" s="18">
         <f>SUM(I22:M22)</f>
         <v/>
       </c>
-      <c r="O22" s="17">
-        <f>M22/$C$5</f>
-        <v/>
-      </c>
-      <c r="P22" s="18">
+      <c r="O22" s="18">
+        <f>M22/$C$5*(1-T22)</f>
+        <v/>
+      </c>
+      <c r="P22" s="19">
         <f>O22*$C$6</f>
         <v/>
       </c>
-      <c r="Q22" s="18">
+      <c r="Q22" s="19">
         <f>O22/(1-$C$7)-O22</f>
         <v/>
       </c>
-      <c r="R22" s="18">
-        <f>O22*$C$8</f>
-        <v/>
-      </c>
-      <c r="S22" s="19">
+      <c r="R22" s="19">
+        <f>IF(T22=0,0,O22/(1-T22)-O22)</f>
+        <v/>
+      </c>
+      <c r="S22" s="20">
         <f>O22+P22+Q22+R22</f>
         <v/>
+      </c>
+      <c r="T22" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1742,7 +1785,7 @@
         <v/>
       </c>
       <c r="O23" s="11">
-        <f>M23/$C$5</f>
+        <f>M23/$C$5*(1-T23)</f>
         <v/>
       </c>
       <c r="P23" s="12">
@@ -1754,89 +1797,95 @@
         <v/>
       </c>
       <c r="R23" s="12">
-        <f>O23*$C$8</f>
+        <f>IF(T23=0,0,O23/(1-T23)-O23)</f>
         <v/>
       </c>
       <c r="S23" s="13">
         <f>O23+P23+Q23+R23</f>
         <v/>
       </c>
+      <c r="T23" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="n">
+      <c r="A24" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>Возмищева Ксения Дмитриевна</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ОРБ)</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>АС</t>
         </is>
       </c>
-      <c r="E24" s="14" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F24" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G24" s="14" t="inlineStr">
+      <c r="G24" s="15" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H24" s="14" t="n">
+      <c r="H24" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I24" s="16" t="n">
+      <c r="I24" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="16" t="n">
+      <c r="J24" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="16" t="n">
+      <c r="K24" s="17" t="n">
         <v>333311.66</v>
       </c>
-      <c r="L24" s="16" t="n">
+      <c r="L24" s="17" t="n">
         <v>1347175.74</v>
       </c>
-      <c r="M24" s="16" t="n">
+      <c r="M24" s="17" t="n">
         <v>1267879.25</v>
       </c>
-      <c r="N24" s="17">
+      <c r="N24" s="18">
         <f>SUM(I24:M24)</f>
         <v/>
       </c>
-      <c r="O24" s="17">
-        <f>M24/$C$5</f>
-        <v/>
-      </c>
-      <c r="P24" s="18">
+      <c r="O24" s="18">
+        <f>M24/$C$5*(1-T24)</f>
+        <v/>
+      </c>
+      <c r="P24" s="19">
         <f>O24*$C$6</f>
         <v/>
       </c>
-      <c r="Q24" s="18">
+      <c r="Q24" s="19">
         <f>O24/(1-$C$7)-O24</f>
         <v/>
       </c>
-      <c r="R24" s="18">
-        <f>O24*$C$8</f>
-        <v/>
-      </c>
-      <c r="S24" s="19">
+      <c r="R24" s="19">
+        <f>IF(T24=0,0,O24/(1-T24)-O24)</f>
+        <v/>
+      </c>
+      <c r="S24" s="20">
         <f>O24+P24+Q24+R24</f>
         <v/>
+      </c>
+      <c r="T24" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="25">
@@ -1896,7 +1945,7 @@
         <v/>
       </c>
       <c r="O25" s="11">
-        <f>M25/$C$5</f>
+        <f>M25/$C$5*(1-T25)</f>
         <v/>
       </c>
       <c r="P25" s="12">
@@ -1908,89 +1957,95 @@
         <v/>
       </c>
       <c r="R25" s="12">
-        <f>O25*$C$8</f>
+        <f>IF(T25=0,0,O25/(1-T25)-O25)</f>
         <v/>
       </c>
       <c r="S25" s="13">
         <f>O25+P25+Q25+R25</f>
         <v/>
       </c>
+      <c r="T25" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="n">
+      <c r="A26" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>Нуруллина Анжелика Альбертовна</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>Fansy</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E26" s="14" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="G26" s="15" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H26" s="14" t="n">
+      <c r="H26" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I26" s="16" t="n">
+      <c r="I26" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="16" t="n">
+      <c r="J26" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="16" t="n">
+      <c r="K26" s="17" t="n">
         <v>338830</v>
       </c>
-      <c r="L26" s="16" t="n">
+      <c r="L26" s="17" t="n">
         <v>1331065</v>
       </c>
-      <c r="M26" s="16" t="n">
+      <c r="M26" s="17" t="n">
         <v>741701</v>
       </c>
-      <c r="N26" s="17">
+      <c r="N26" s="18">
         <f>SUM(I26:M26)</f>
         <v/>
       </c>
-      <c r="O26" s="17">
-        <f>M26/$C$5</f>
-        <v/>
-      </c>
-      <c r="P26" s="18">
+      <c r="O26" s="18">
+        <f>M26/$C$5*(1-T26)</f>
+        <v/>
+      </c>
+      <c r="P26" s="19">
         <f>O26*$C$6</f>
         <v/>
       </c>
-      <c r="Q26" s="18">
+      <c r="Q26" s="19">
         <f>O26/(1-$C$7)-O26</f>
         <v/>
       </c>
-      <c r="R26" s="18">
-        <f>O26*$C$8</f>
-        <v/>
-      </c>
-      <c r="S26" s="19">
+      <c r="R26" s="19">
+        <f>IF(T26=0,0,O26/(1-T26)-O26)</f>
+        <v/>
+      </c>
+      <c r="S26" s="20">
         <f>O26+P26+Q26+R26</f>
         <v/>
+      </c>
+      <c r="T26" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="27">
@@ -2050,7 +2105,7 @@
         <v/>
       </c>
       <c r="O27" s="11">
-        <f>M27/$C$5</f>
+        <f>M27/$C$5*(1-T27)</f>
         <v/>
       </c>
       <c r="P27" s="12">
@@ -2062,89 +2117,95 @@
         <v/>
       </c>
       <c r="R27" s="12">
-        <f>O27*$C$8</f>
+        <f>IF(T27=0,0,O27/(1-T27)-O27)</f>
         <v/>
       </c>
       <c r="S27" s="13">
         <f>O27+P27+Q27+R27</f>
         <v/>
       </c>
+      <c r="T27" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="n">
+      <c r="A28" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Лукьянова Вера Константиновна</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ПО)</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E28" s="14" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G28" s="14" t="inlineStr">
+      <c r="G28" s="15" t="inlineStr">
         <is>
           <t>2024–2026</t>
         </is>
       </c>
-      <c r="H28" s="14" t="n">
+      <c r="H28" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I28" s="16" t="n">
+      <c r="I28" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J28" s="16" t="n">
+      <c r="J28" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="16" t="n">
+      <c r="K28" s="17" t="n">
         <v>141702</v>
       </c>
-      <c r="L28" s="16" t="n">
+      <c r="L28" s="17" t="n">
         <v>73617</v>
       </c>
-      <c r="M28" s="16" t="n">
+      <c r="M28" s="17" t="n">
         <v>973404</v>
       </c>
-      <c r="N28" s="17">
+      <c r="N28" s="18">
         <f>SUM(I28:M28)</f>
         <v/>
       </c>
-      <c r="O28" s="17">
-        <f>M28/$C$5</f>
-        <v/>
-      </c>
-      <c r="P28" s="18">
+      <c r="O28" s="18">
+        <f>M28/$C$5*(1-T28)</f>
+        <v/>
+      </c>
+      <c r="P28" s="19">
         <f>O28*$C$6</f>
         <v/>
       </c>
-      <c r="Q28" s="18">
+      <c r="Q28" s="19">
         <f>O28/(1-$C$7)-O28</f>
         <v/>
       </c>
-      <c r="R28" s="18">
-        <f>O28*$C$8</f>
-        <v/>
-      </c>
-      <c r="S28" s="19">
+      <c r="R28" s="19">
+        <f>IF(T28=0,0,O28/(1-T28)-O28)</f>
+        <v/>
+      </c>
+      <c r="S28" s="20">
         <f>O28+P28+Q28+R28</f>
         <v/>
+      </c>
+      <c r="T28" s="14" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="29">
@@ -2204,7 +2265,7 @@
         <v/>
       </c>
       <c r="O29" s="11">
-        <f>M29/$C$5</f>
+        <f>M29/$C$5*(1-T29)</f>
         <v/>
       </c>
       <c r="P29" s="12">
@@ -2216,194 +2277,200 @@
         <v/>
       </c>
       <c r="R29" s="12">
-        <f>O29*$C$8</f>
+        <f>IF(T29=0,0,O29/(1-T29)-O29)</f>
         <v/>
       </c>
       <c r="S29" s="13">
         <f>O29+P29+Q29+R29</f>
         <v/>
       </c>
+      <c r="T29" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="n">
+      <c r="A30" s="15" t="n">
         <v>20</v>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>Капустина Вероника Сергеевна</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>ТФМ (ОСК)</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>БВ</t>
         </is>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>6%</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="F30" s="15" t="inlineStr">
         <is>
           <t>активен</t>
         </is>
       </c>
-      <c r="G30" s="14" t="inlineStr">
+      <c r="G30" s="15" t="inlineStr">
         <is>
           <t>2025–2026</t>
         </is>
       </c>
-      <c r="H30" s="14" t="n">
+      <c r="H30" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="I30" s="16" t="n">
+      <c r="I30" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="J30" s="16" t="n">
+      <c r="J30" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="K30" s="16" t="n">
+      <c r="K30" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="L30" s="16" t="n">
+      <c r="L30" s="17" t="n">
         <v>214440.3</v>
       </c>
-      <c r="M30" s="16" t="n">
+      <c r="M30" s="17" t="n">
         <v>1228052.73</v>
       </c>
-      <c r="N30" s="17">
+      <c r="N30" s="18">
         <f>SUM(I30:M30)</f>
         <v/>
       </c>
-      <c r="O30" s="17">
-        <f>M30/$C$5</f>
-        <v/>
-      </c>
-      <c r="P30" s="18">
+      <c r="O30" s="18">
+        <f>M30/$C$5*(1-T30)</f>
+        <v/>
+      </c>
+      <c r="P30" s="19">
         <f>O30*$C$6</f>
         <v/>
       </c>
-      <c r="Q30" s="18">
+      <c r="Q30" s="19">
         <f>O30/(1-$C$7)-O30</f>
         <v/>
       </c>
-      <c r="R30" s="18">
-        <f>O30*$C$8</f>
-        <v/>
-      </c>
-      <c r="S30" s="19">
+      <c r="R30" s="19">
+        <f>IF(T30=0,0,O30/(1-T30)-O30)</f>
+        <v/>
+      </c>
+      <c r="S30" s="20">
         <f>O30+P30+Q30+R30</f>
         <v/>
       </c>
+      <c r="T30" s="14" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="n"/>
-      <c r="B31" s="21" t="inlineStr">
+      <c r="A31" s="21" t="n"/>
+      <c r="B31" s="22" t="inlineStr">
         <is>
           <t>ИТОГО (20 чел.)</t>
         </is>
       </c>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="20" t="n"/>
-      <c r="E31" s="20" t="n"/>
-      <c r="F31" s="20" t="n"/>
-      <c r="G31" s="20" t="n"/>
-      <c r="H31" s="20" t="n"/>
-      <c r="I31" s="22">
+      <c r="C31" s="21" t="n"/>
+      <c r="D31" s="21" t="n"/>
+      <c r="E31" s="21" t="n"/>
+      <c r="F31" s="21" t="n"/>
+      <c r="G31" s="21" t="n"/>
+      <c r="H31" s="21" t="n"/>
+      <c r="I31" s="23">
         <f>SUM(I11:I30)</f>
         <v/>
       </c>
-      <c r="J31" s="22">
+      <c r="J31" s="23">
         <f>SUM(J11:J30)</f>
         <v/>
       </c>
-      <c r="K31" s="22">
+      <c r="K31" s="23">
         <f>SUM(K11:K30)</f>
         <v/>
       </c>
-      <c r="L31" s="22">
+      <c r="L31" s="23">
         <f>SUM(L11:L30)</f>
         <v/>
       </c>
-      <c r="M31" s="22">
+      <c r="M31" s="23">
         <f>SUM(M11:M30)</f>
         <v/>
       </c>
-      <c r="N31" s="22">
+      <c r="N31" s="23">
         <f>SUM(N11:N30)</f>
         <v/>
       </c>
-      <c r="O31" s="22">
+      <c r="O31" s="23">
         <f>SUM(O11:O30)</f>
         <v/>
       </c>
-      <c r="P31" s="22">
+      <c r="P31" s="23">
         <f>SUM(P11:P30)</f>
         <v/>
       </c>
-      <c r="Q31" s="22">
+      <c r="Q31" s="23">
         <f>SUM(Q11:Q30)</f>
         <v/>
       </c>
-      <c r="R31" s="22">
+      <c r="R31" s="23">
         <f>SUM(R11:R30)</f>
         <v/>
       </c>
-      <c r="S31" s="22">
+      <c r="S31" s="23">
         <f>SUM(S11:S30)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="23" t="inlineStr">
+      <c r="A33" s="24" t="inlineStr">
         <is>
           <t>ПЛАНИРОВАНИЕ</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="25" t="inlineStr">
         <is>
           <t>Месячный фонд (итого к оплате)</t>
         </is>
       </c>
-      <c r="B34" s="25" t="inlineStr"/>
-      <c r="C34" s="26">
+      <c r="B34" s="26" t="inlineStr"/>
+      <c r="C34" s="27">
         <f>S31*1</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="24" t="inlineStr">
+      <c r="A35" s="25" t="inlineStr">
         <is>
           <t>На 6 месяцев</t>
         </is>
       </c>
-      <c r="B35" s="25" t="inlineStr"/>
-      <c r="C35" s="26">
+      <c r="B35" s="26" t="inlineStr"/>
+      <c r="C35" s="27">
         <f>S31*6</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="24" t="inlineStr">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>На 12 месяцев</t>
         </is>
       </c>
-      <c r="B36" s="25" t="inlineStr"/>
-      <c r="C36" s="26">
+      <c r="B36" s="26" t="inlineStr"/>
+      <c r="C36" s="27">
         <f>S31*12</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="27" t="inlineStr">
+      <c r="A38" s="28" t="inlineStr">
         <is>
           <t>Примечания</t>
         </is>
@@ -2433,28 +2500,28 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>4. Среднемесячная выплата 2026 = «Итого 2026» ÷ C5. Это фактический месячный run-rate по начислениям декабрь 2025 – июнь 2026.</t>
+          <t>4. Среднемес. «на руки» 2026 = «Итого 2026» ÷ C5 × (1 − ставка НПД). В исходнике «Итого к выплате» = «на руки» ÷ (1 − ставка), проверено: 236 756 ÷ 0,94 = 251 868.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>5. ВАЖНО: базовая сумма — «Итого к выплате», она УЖЕ включает НПД. Столбец «С НПД +6%» начисляет налог поверх этой суммы. Если нужен НПД на сумму «на руки», базу надо заменить.</t>
+          <t>5. База расчёта — сумма «на руки» (без НПД). Столбцы 2022–2026 и «Итого 2022–2026» остались в «Итого к выплате» — это данные исходника.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>6. Все три надбавки считаются от среднемесячной выплаты: комиссия 4dev = ×3%; сбор ЮЛ Сингапура = ÷0,975 − среднемесячная (2,5% сверху); НПД = ×6%.</t>
+          <t>6. Надбавки от «на руки»: комиссия 4dev = ×3%; сбор ЮЛ Сингапура = ÷0,975 − база; НПД = ÷(1 − ставка) − база, т.е. так же, как считает исходный файл.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>7. «ИТОГО к оплате в месяц» = среднемесячная + комиссия + сбор + НПД (надбавки не каскадируются). Если применять их последовательно (÷0,975 × 1,06 × 1,03), итог по группе будет 3 830 014 ₽ вместо 3 815 806 ₽.</t>
+          <t>7. «ИТОГО к оплате в месяц» = на руки + комиссия + сбор + НПД (надбавки не каскадируются). Столбец T — ставка НПД по каждому человеку (у Абдуллиной 0%).</t>
         </is>
       </c>
     </row>

</xml_diff>